<commit_message>
Added row of samples
</commit_message>
<xml_diff>
--- a/Palacios_Ex3A_tables.xlsx
+++ b/Palacios_Ex3A_tables.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charlespalacios\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7EAF457B-281C-4A83-892B-050207C87100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{0FF7760E-DF3A-4679-A755-1A9B02586755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="2" activeTab="4" xr2:uid="{5DD4051D-997A-4BA5-B704-E1C3CD18D9D8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="4" xr2:uid="{5DD4051D-997A-4BA5-B704-E1C3CD18D9D8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Customer" sheetId="1" r:id="rId1"/>
-    <sheet name="Dog" sheetId="2" r:id="rId2"/>
-    <sheet name="Walk" sheetId="3" r:id="rId3"/>
-    <sheet name="Employee" sheetId="4" r:id="rId4"/>
-    <sheet name="Payment" sheetId="5" r:id="rId5"/>
+    <sheet name="customers" sheetId="1" r:id="rId1"/>
+    <sheet name="dogs" sheetId="2" r:id="rId2"/>
+    <sheet name="walkers" sheetId="4" r:id="rId3"/>
+    <sheet name="walks" sheetId="3" r:id="rId4"/>
+    <sheet name="payments" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,88 +40,183 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
-  <si>
-    <t xml:space="preserve">CustomerID </t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
-    <t>EmergencyContact</t>
-  </si>
-  <si>
-    <t>DogID</t>
-  </si>
-  <si>
-    <t>CustomerID</t>
-  </si>
-  <si>
-    <t>Breed</t>
-  </si>
-  <si>
-    <t>Age</t>
-  </si>
-  <si>
-    <t>Size</t>
-  </si>
-  <si>
-    <t>Medical/Behavorial Notes</t>
-  </si>
-  <si>
-    <t>Weight</t>
-  </si>
-  <si>
-    <t>WalkID</t>
-  </si>
-  <si>
-    <t>EmployeeID</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Time</t>
-  </si>
-  <si>
-    <t>Duration</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>HireDate</t>
-  </si>
-  <si>
-    <t>PaymentID</t>
-  </si>
-  <si>
-    <t>Amount</t>
-  </si>
-  <si>
-    <t>Method</t>
-  </si>
-  <si>
-    <t>Status</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="52">
+  <si>
+    <t xml:space="preserve">customer_id </t>
+  </si>
+  <si>
+    <t>first_name</t>
+  </si>
+  <si>
+    <t>last_name</t>
+  </si>
+  <si>
+    <t>phone</t>
+  </si>
+  <si>
+    <t>email</t>
+  </si>
+  <si>
+    <t>address</t>
+  </si>
+  <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>state</t>
+  </si>
+  <si>
+    <t>emergency_contact</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>dog_id</t>
+  </si>
+  <si>
+    <t>customer_id</t>
+  </si>
+  <si>
+    <t>dog_name</t>
+  </si>
+  <si>
+    <t>breed</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>size</t>
+  </si>
+  <si>
+    <t>walker_id</t>
+  </si>
+  <si>
+    <t>walk_id`</t>
+  </si>
+  <si>
+    <t>sheduled_date</t>
+  </si>
+  <si>
+    <t>scheduled_time</t>
+  </si>
+  <si>
+    <t>duration_minutes</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>completion_time</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>payment_id</t>
+  </si>
+  <si>
+    <t>walk_id</t>
+  </si>
+  <si>
+    <t>amount</t>
+  </si>
+  <si>
+    <t>payment_date</t>
+  </si>
+  <si>
+    <t>payment_method</t>
+  </si>
+  <si>
+    <t>payment_status</t>
+  </si>
+  <si>
+    <t>571-322-1253</t>
+  </si>
+  <si>
+    <t>charpal@email.com</t>
+  </si>
+  <si>
+    <t>123 Ash Rd</t>
+  </si>
+  <si>
+    <t>Coolsville</t>
+  </si>
+  <si>
+    <t>Char</t>
+  </si>
+  <si>
+    <t>Pal</t>
+  </si>
+  <si>
+    <t>VA</t>
+  </si>
+  <si>
+    <t>Jenn Pal - 703-989-0129</t>
+  </si>
+  <si>
+    <t>Char asks if we can call him if anything were to happen</t>
+  </si>
+  <si>
+    <t>Mandoor</t>
+  </si>
+  <si>
+    <t>Pekingnese</t>
+  </si>
+  <si>
+    <t>Small</t>
+  </si>
+  <si>
+    <t>Fights when trying to put the leash on her</t>
+  </si>
+  <si>
+    <t>Lana</t>
+  </si>
+  <si>
+    <t>Jones</t>
+  </si>
+  <si>
+    <t>571-321-4214</t>
+  </si>
+  <si>
+    <t>ljones@lanadogwalking.com</t>
+  </si>
+  <si>
+    <t>0 hr 25 min</t>
+  </si>
+  <si>
+    <t>complete</t>
+  </si>
+  <si>
+    <t>Good walk, Mandoor did slip out of her leash though, I suggest getting a tighter leash</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>PAID</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="6" formatCode="&quot;$&quot;#,##0_);[Red]\(&quot;$&quot;#,##0\)"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -162,16 +257,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="18" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="6" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -504,14 +605,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{64EBA36B-59EB-4237-9301-1BD2B941DC7B}">
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="3.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="44.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -530,51 +639,118 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>110</v>
+      </c>
+      <c r="B2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D2" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" t="s">
+        <v>36</v>
+      </c>
+      <c r="I2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J2" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{631D6173-6528-44F3-9500-79BFBEF667D9}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{571C5799-1E0C-432A-8F77-72C66520B74D}">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.21875" customWidth="1"/>
-    <col min="7" max="7" width="6.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="5.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D1" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E1" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" t="s">
+        <v>15</v>
+      </c>
+      <c r="G1" t="s">
         <v>9</v>
       </c>
-      <c r="F1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
         <v>11</v>
+      </c>
+      <c r="B2">
+        <v>110</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D2" t="s">
+        <v>40</v>
+      </c>
+      <c r="E2">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G2" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -583,70 +759,136 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47F4D1A1-E9AE-4867-9DDB-C39E99B60481}">
-  <dimension ref="A1:G1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21A2E1C-880C-4A72-AE15-587268A3D7F7}">
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F1" t="s">
-        <v>17</v>
-      </c>
-      <c r="G1" t="s">
-        <v>18</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D2" t="s">
+        <v>45</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E2" r:id="rId1" xr:uid="{FE1D64AE-47E1-4988-8B6A-2DFB62EEC43D}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21A2E1C-880C-4A72-AE15-587268A3D7F7}">
-  <dimension ref="A1:E1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47F4D1A1-E9AE-4867-9DDB-C39E99B60481}">
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="67.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
+        <v>17</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>18</v>
       </c>
       <c r="E1" t="s">
         <v>19</v>
+      </c>
+      <c r="F1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>111</v>
+      </c>
+      <c r="C2">
+        <v>101</v>
+      </c>
+      <c r="D2" s="5">
+        <v>46113</v>
+      </c>
+      <c r="E2" s="6">
+        <v>0.54166666666666663</v>
+      </c>
+      <c r="F2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H2" s="6">
+        <v>0.55902777777777779</v>
+      </c>
+      <c r="I2" s="7">
+        <v>25</v>
+      </c>
+      <c r="J2" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
@@ -656,39 +898,62 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A19D203-4663-4E31-9AB3-255E2A331C3A}">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="7.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="7" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="6" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="D1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="E1" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="F1" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="G1" t="s">
-        <v>23</v>
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1000</v>
+      </c>
+      <c r="B2">
+        <v>110</v>
+      </c>
+      <c r="C2">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7">
+        <v>25</v>
+      </c>
+      <c r="E2" s="5">
+        <v>46112</v>
+      </c>
+      <c r="F2" t="s">
+        <v>50</v>
+      </c>
+      <c r="G2" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>